<commit_message>
fonctionnalite : ajouter le premier probleme rencontre
</commit_message>
<xml_diff>
--- a/Mon Feuille de Calcul.xlsx
+++ b/Mon Feuille de Calcul.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AWS ODC\Probleme_Resolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDA63FE0-5CA5-4034-A496-89C33E787257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D83154C-5F86-4067-83B6-55EC0DAC16F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
   <sheets>
     <sheet name="Base de connaissance vierge(Ent" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Problème n°</t>
   </si>
@@ -44,13 +44,50 @@
   </si>
   <si>
     <t>Commentaires</t>
+  </si>
+  <si>
+    <t>n° :
+1</t>
+  </si>
+  <si>
+    <t>AWS / Auto Scaling / IAM</t>
+  </si>
+  <si>
+    <t>Erreur lors de la création d’une politique 
+de mise à l’échelle pour un groupe Auto Scaling EC2.
+ Le service indique que le rôle lié 
+au service n’est pas encore disponible.</t>
+  </si>
+  <si>
+    <t>Message d’erreur lors de la création de la politique de scaling
+Mention : “EC2 Auto Scaling n'a pas l'autorisation…”
+Groupe Auto Scaling créé avec succès mais scaling policy échoue</t>
+  </si>
+  <si>
+    <t>Le rôle IAM lié au service (Service-Linked Role) pour Auto Scaling n’est pas encore propagé ou disponible au moment de la création de la politique. AWS nécessite un délai pour rendre les nouveaux rôles utilisables.</t>
+  </si>
+  <si>
+    <t>Attendre quelques minutes (1 à 5 min) pour la propagation du rôle
+Rafraîchir la console AWS
+Recréer la politique de scaling
+Vérifier que le rôle AWSServiceRoleForAutoScaling existe dans IAM
+Si absent, recréer le rôle ou relancer la création du groupe</t>
+  </si>
+  <si>
+    <t>AWS IAM Console
+AWS EC2 Auto Scaling
+CloudTrail (pour vérifier les erreurs)
+Documentation AWS (Service-linked roles)</t>
+  </si>
+  <si>
+    <t>Problème temporaire courant lié à la propagation IAM. Ne nécessite généralement pas d’intervention avancée.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +218,21 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -533,9 +585,21 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -891,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87A119-DF5E-4ED7-A85D-3E01B73E9539}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" customWidth="1"/>
@@ -931,6 +995,32 @@
       </c>
       <c r="I1" s="1"/>
     </row>
+    <row r="2" spans="1:9" ht="186" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
maintenance : mettre a jour la feuille de calcul
</commit_message>
<xml_diff>
--- a/Mon Feuille de Calcul.xlsx
+++ b/Mon Feuille de Calcul.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AWS ODC\Probleme_Resolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D83154C-5F86-4067-83B6-55EC0DAC16F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0259FE4-660A-4782-A736-B8CA332A4D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Problème n°</t>
   </si>
@@ -44,10 +44,6 @@
   </si>
   <si>
     <t>Commentaires</t>
-  </si>
-  <si>
-    <t>n° :
-1</t>
   </si>
   <si>
     <t>AWS / Auto Scaling / IAM</t>
@@ -81,6 +77,46 @@
   </si>
   <si>
     <t>Problème temporaire courant lié à la propagation IAM. Ne nécessite généralement pas d’intervention avancée.</t>
+  </si>
+  <si>
+    <t>Télécharger la policy IAM lab_policy en
+ JSON via AWS CLI (sans utiliser la console).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° :2 Téléchargement d’une policy IAM via AWS CLI
+</t>
+  </si>
+  <si>
+    <t>N° :1  AWS Auto Scaling n’a pas encore les permissions nécessaires pour fonctionner</t>
+  </si>
+  <si>
+    <t>Récupérer une policy IAM (lab_policy) 
+en JSON sans utiliser la console AWS.</t>
+  </si>
+  <si>
+    <t>Message d’erreur lors de l’exécution de la commande :
+Invalid length for parameter PolicyArn
+Message indiquant un paramètre manquant :
+the following arguments are required: --version-id
+Impossible de récupérer le document JSON de la policy</t>
+  </si>
+  <si>
+    <t>Mauvais ARN utilisé (placeholder)
+Oubli du paramètre obligatoire --version-id</t>
+  </si>
+  <si>
+    <t>Lister les policies avec aws iam list-policies --scope Local
+Récupérer l’ARN de la policy
+Obtenir la version avec aws iam get-policy
+Télécharger la policy avec aws iam get-policy-version
+Rediriger la sortie vers un fichier JSON avec &gt;</t>
+  </si>
+  <si>
+    <t>AWS CLI
+Documentation IAM CLI</t>
+  </si>
+  <si>
+    <t>Respecter les paramètres obligatoires et utiliser le bon ARN.</t>
   </si>
 </sst>
 </file>
@@ -585,7 +621,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -599,6 +635,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -955,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87A119-DF5E-4ED7-A85D-3E01B73E9539}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" customWidth="1"/>
@@ -997,28 +1036,54 @@
     </row>
     <row r="2" spans="1:9" ht="186" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="186" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mise a jour de la feuille de calcul
</commit_message>
<xml_diff>
--- a/Mon Feuille de Calcul.xlsx
+++ b/Mon Feuille de Calcul.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AWS ODC\Probleme_Resolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0259FE4-660A-4782-A736-B8CA332A4D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EDCC08-7D25-46C4-ACDC-BA82A7ED111A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Problème n°</t>
   </si>
@@ -117,6 +117,30 @@
   </si>
   <si>
     <t>Respecter les paramètres obligatoires et utiliser le bon ARN.</t>
+  </si>
+  <si>
+    <t>N°:3 Lambda timeout et connexion à la base de donnees</t>
+  </si>
+  <si>
+    <t>AWS / Lambda / RDS / VPC / IAM / SNS</t>
+  </si>
+  <si>
+    <t>Pendant le TP, la fonction Lambda n’arrivait pas à se connecter à la base de donnees ni à recuperer certains parametres, ce qui bloquait tout le traitement.</t>
+  </si>
+  <si>
+    <t>La Lambda finissait en timeout, parfois avec AccessDenied, aucun email n’etait envoye via SNS, et selon les essais on voyait aussi des erreurs de handler ou de module manquant dans CloudWatch.</t>
+  </si>
+  <si>
+    <t>La fonction etait dans un VPC mal configure : sous-reseaux sans sortie correcte, groupe de securite qui ne laissait pas passer le port de la base, et quelques permissions IAM manquaient pour lire les parametres ou publier le message. Dans certains cas, le handler ou le package deploye n’etaient pas corrects.</t>
+  </si>
+  <si>
+    <t>Verifier d’abord la connectivite reseau entre Lambda et la base : meme VPC ou routage correct, bon security group et port ouvert. Ajouter les autorisations IAM necessaires pour lire Parameter Store et publier vers SNS. Controler ensuite le nom du handler, les dependances incluses dans le zip ou le layer, puis relancer des tests avec CloudWatch Logs pour valider chaque etape.</t>
+  </si>
+  <si>
+    <t>Lambda, RDS, VPC, Security Groups, IAM, SNS, CloudWatch Logs</t>
+  </si>
+  <si>
+    <t>Probleme rencontre en plusieurs etapes du TP ; il venait souvent de plusieurs petites erreurs en meme temps, pas d’une seule cause.</t>
   </si>
 </sst>
 </file>
@@ -994,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87A119-DF5E-4ED7-A85D-3E01B73E9539}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" customWidth="1"/>
@@ -1086,6 +1110,32 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:9" ht="232" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ajouter de nouvelles entrees dans la feuille de calcul
</commit_message>
<xml_diff>
--- a/Mon Feuille de Calcul.xlsx
+++ b/Mon Feuille de Calcul.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AWS ODC\Probleme_Resolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EDCC08-7D25-46C4-ACDC-BA82A7ED111A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC21512-A73A-45F9-9254-3C87B498FB4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="71">
   <si>
     <t>Problème n°</t>
   </si>
@@ -141,6 +141,146 @@
   </si>
   <si>
     <t>Probleme rencontre en plusieurs etapes du TP ; il venait souvent de plusieurs petites erreurs en meme temps, pas d’une seule cause.</t>
+  </si>
+  <si>
+    <t>AWS / EC2 / Web Server</t>
+  </si>
+  <si>
+    <t>Le serveur web EC2 était installé mais aucune page web par défaut (index.html) n’était présente, empéchant l’affichage du site via le DNS public</t>
+  </si>
+  <si>
+    <t>Accés au DNS public affiche une page vide ou une erreur malgré une instance en cours d’éxécution</t>
+  </si>
+  <si>
+    <t>Le service web fonctionnait correctement mais aucun contenu n’était présent dans le répertoire /var/www/html, donc rien à afficher</t>
+  </si>
+  <si>
+    <t>Connexion en SSH à l’instance EC2
+Création d’un fichier index.html dans /var/www/html
+Redémarrage du service httpd
+Test avec curl puis navigateur</t>
+  </si>
+  <si>
+    <t>EC2 Console
+SSH
+Apache
+curl</t>
+  </si>
+  <si>
+    <t>Probléme simple de configuration lié à l’absence de contenu web, résolu rapidement</t>
+  </si>
+  <si>
+    <t>N° : 4  L’absence de fichier index.html (page web par défaut) dans le serveur web, empêchant l’affichage du site.</t>
+  </si>
+  <si>
+    <t>N° : 5 – AMI invalide</t>
+  </si>
+  <si>
+    <t>AWS / EC2 / CLI</t>
+  </si>
+  <si>
+    <t>L’ID de l’AMI utilisé dans le script était invalide pour la région sélectionnée, empêchant la création de l’instance EC2</t>
+  </si>
+  <si>
+    <t>Erreur « InvalidAMIID.NotFound » lors de l’exécution du script</t>
+  </si>
+  <si>
+    <t>Mauvaise correspondance entre l’AMI et la région AWS utilisée dans la commande run-instances</t>
+  </si>
+  <si>
+    <t>Analyse du script bash
+Vérification de la région AWS
+Correction de l’AMI
+Relance du script</t>
+  </si>
+  <si>
+    <t>AWS CLI
+Script bash
+EC2 Console</t>
+  </si>
+  <si>
+    <t>Problème de configuration lié aux régions AWS</t>
+  </si>
+  <si>
+    <t>N° : 6 – Port HTTP fermé</t>
+  </si>
+  <si>
+    <t>AWS / EC2 / Réseau</t>
+  </si>
+  <si>
+    <t>Le port HTTP (80) n’était pas ouvert dans le Security Group, empêchant l’accès au serveur web</t>
+  </si>
+  <si>
+    <t>Impossible d’accéder à la page web via l’IP publique</t>
+  </si>
+  <si>
+    <t>Absence de règle entrante autorisant le trafic HTTP</t>
+  </si>
+  <si>
+    <t>Vérification avec nmap
+Modification du Security Group
+Ajout règle HTTP (port 80)</t>
+  </si>
+  <si>
+    <t>nmap
+EC2 Console
+Security Groups</t>
+  </si>
+  <si>
+    <t>Problème réseau classique</t>
+  </si>
+  <si>
+    <t>N° : 7 – Service Apache arrêté</t>
+  </si>
+  <si>
+    <t>AWS / EC2 / Service</t>
+  </si>
+  <si>
+    <t>Le service Apache (httpd) n’était pas démarré après le lancement de l’instance</t>
+  </si>
+  <si>
+    <t>Page web inaccessible malgré port ouvert</t>
+  </si>
+  <si>
+    <t>Le service web n’était pas actif sur l’instance</t>
+  </si>
+  <si>
+    <t>Connexion SSH
+Vérification avec systemctl
+Démarrage et activation du service</t>
+  </si>
+  <si>
+    <t>SSH
+systemctl
+Apache</t>
+  </si>
+  <si>
+    <t>Problème lié aux services Linux</t>
+  </si>
+  <si>
+    <t>N° : 8 – Absence de page web</t>
+  </si>
+  <si>
+    <t>Le serveur web était installé mais aucune page index.html n’était présente</t>
+  </si>
+  <si>
+    <t>Page vide ou erreur lors de l’accès via navigateur</t>
+  </si>
+  <si>
+    <t>Aucun contenu dans /var/www/html</t>
+  </si>
+  <si>
+    <t>Création d’un fichier index.html
+Redémarrage du service
+Test navigateur</t>
+  </si>
+  <si>
+    <t>SSH
+Apache
+curl</t>
+  </si>
+  <si>
+    <t>Problème simple de configuration</t>
   </si>
 </sst>
 </file>
@@ -298,7 +438,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -481,6 +621,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -645,9 +791,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -657,11 +802,15 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1018,10 +1167,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87A119-DF5E-4ED7-A85D-3E01B73E9539}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.6328125" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="29.453125" customWidth="1"/>
     <col min="4" max="4" width="24.81640625" customWidth="1"/>
@@ -1031,109 +1180,239 @@
     <col min="8" max="8" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1"/>
+      <c r="I1" s="5"/>
     </row>
     <row r="2" spans="1:9" ht="186" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="186" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="232" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="4" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corriger le classeur Excel et ajouter le probleme numero 9
</commit_message>
<xml_diff>
--- a/Mon Feuille de Calcul.xlsx
+++ b/Mon Feuille de Calcul.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AWS ODC\Probleme_Resolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC21512-A73A-45F9-9254-3C87B498FB4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E49441-58DE-40E9-96B5-2C6F46CC2FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
   <si>
     <t>Problème n°</t>
   </si>
@@ -282,12 +282,41 @@
   <si>
     <t>Problème simple de configuration</t>
   </si>
+  <si>
+    <t>N° : 9 – Upload inefficace avec aws s3 cp</t>
+  </si>
+  <si>
+    <t>AWS / S3 / CLI</t>
+  </si>
+  <si>
+    <t>Le script utilisait la commande aws s3 cp, ce qui rechargeait tous les fichiers du site à chaque exécution même sans modification.</t>
+  </si>
+  <si>
+    <t>Temps de chargement plus long et transfert inutile de fichiers non modifiés vers le bucket S3.</t>
+  </si>
+  <si>
+    <t>La commande aws s3 cp ne vérifie pas les différences entre les fichiers locaux et ceux déjà présents dans S3.</t>
+  </si>
+  <si>
+    <t>Modification du fichier index.html pour tester
+Remplacement de la commande aws s3 cp par aws s3 sync
+Exécution du script mis à jour
+Vérification des fichiers uploadés</t>
+  </si>
+  <si>
+    <t>AWS CLI
+Amazon S3
+Terminal SSH</t>
+  </si>
+  <si>
+    <t>La commande aws s3 sync est plus efficace car elle ne met à jour que les fichiers modifiés, comme index.html, contrairement à aws s3 cp qui recharge tous les fichiers.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -424,21 +453,36 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -630,8 +674,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -746,6 +796,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -791,26 +856,27 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1167,252 +1233,279 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87A119-DF5E-4ED7-A85D-3E01B73E9539}">
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" customWidth="1"/>
-    <col min="2" max="2" width="35" customWidth="1"/>
-    <col min="3" max="3" width="29.453125" customWidth="1"/>
-    <col min="4" max="4" width="24.81640625" customWidth="1"/>
-    <col min="5" max="5" width="35.08984375" customWidth="1"/>
-    <col min="6" max="6" width="24.90625" customWidth="1"/>
-    <col min="7" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="23" customWidth="1"/>
+    <col min="1" max="1" width="24.6328125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="35" style="2" customWidth="1"/>
+    <col min="3" max="3" width="43.6328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="29.36328125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="35.08984375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="33.54296875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="29.54296875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="23" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="10.90625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5"/>
+      <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9" ht="186" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:9" ht="252" x14ac:dyDescent="0.5">
+      <c r="A2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="186" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:9" ht="273" x14ac:dyDescent="0.5">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="232" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:9" ht="336" x14ac:dyDescent="0.5">
+      <c r="A4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="7" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="186" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A10" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corriger l ouverture du classeur Excel et ajouter les problemes 10 et 11
</commit_message>
<xml_diff>
--- a/Mon Feuille de Calcul.xlsx
+++ b/Mon Feuille de Calcul.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\AWS ODC\Probleme_Resolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E49441-58DE-40E9-96B5-2C6F46CC2FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5C81759-1327-49EB-8CE9-F00CF08218EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="95">
   <si>
     <t>Problème n°</t>
   </si>
@@ -311,12 +311,69 @@
   <si>
     <t>La commande aws s3 sync est plus efficace car elle ne met à jour que les fichiers modifiés, comme index.html, contrairement à aws s3 cp qui recharge tous les fichiers.</t>
   </si>
+  <si>
+    <t>N° : 10 – Problème de permissions et configuration SNS</t>
+  </si>
+  <si>
+    <t>AWS / Lambda / IAM / SNS</t>
+  </si>
+  <si>
+    <t>La fonction Lambda ne pouvait pas envoyer le résultat par e-mail en raison de permissions insuffisantes ou d'une mauvaise configuration du topic SNS</t>
+  </si>
+  <si>
+    <t>Aucun e-mail reçu après upload du fichier dans S3</t>
+  </si>
+  <si>
+    <t>Rôle IAM incomplet, ARN SNS incorrect ou abonnement non confirmé</t>
+  </si>
+  <si>
+    <t>Vérification du rôle LambdaAccessRole
+Correction de l'ARN SNS
+Confirmation de l'abonnement e-mail</t>
+  </si>
+  <si>
+    <t>AWS IAM
+SNS
+Lambda</t>
+  </si>
+  <si>
+    <t>Problème critique lié à la sécurité et à la configuration des services AWS</t>
+  </si>
+  <si>
+    <t>N° : 11 – Déclenchement et traitement du fichier S3</t>
+  </si>
+  <si>
+    <t>AWS / Lambda / S3</t>
+  </si>
+  <si>
+    <t>La fonction Lambda ne se déclenchait pas ou ne traitait pas correctement le fichier texte chargé dans S3</t>
+  </si>
+  <si>
+    <t>Aucun traitement ou nombre de mots incorrect</t>
+  </si>
+  <si>
+    <t>Absence de trigger S3, fichier mal formaté ou erreur dans le code de lecture du fichier</t>
+  </si>
+  <si>
+    <t>Ajout du trigger S3 (PUT)
+Vérification du format du fichier .txt
+Correction du code Python pour lire et compter les mots</t>
+  </si>
+  <si>
+    <t>S3
+Lambda
+Python
+CloudWatch Logs</t>
+  </si>
+  <si>
+    <t>Problème lié à l'intégration entre services et au traitement des données</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,8 +538,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -677,6 +749,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF333F4F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -856,27 +940,24 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1233,7 +1314,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C87A119-DF5E-4ED7-A85D-3E01B73E9539}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="24.6328125" style="2" customWidth="1"/>
@@ -1247,265 +1328,317 @@
     <col min="9" max="16384" width="10.90625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:9" ht="42" x14ac:dyDescent="0.5">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="252" x14ac:dyDescent="0.5">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="273" x14ac:dyDescent="0.5">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="336" x14ac:dyDescent="0.5">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:9" ht="189" x14ac:dyDescent="0.5">
+      <c r="A5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:9" ht="105" x14ac:dyDescent="0.5">
+      <c r="A6" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:9" ht="84" x14ac:dyDescent="0.5">
+      <c r="A7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:9" ht="84" x14ac:dyDescent="0.5">
+      <c r="A8" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="139" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:9" ht="84" x14ac:dyDescent="0.5">
+      <c r="A9" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="186" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:9" ht="231" x14ac:dyDescent="0.5">
+      <c r="A10" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="3" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="105" x14ac:dyDescent="0.5">
+      <c r="A11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="126" x14ac:dyDescent="0.5">
+      <c r="A12" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>